<commit_message>
Added more options for management
</commit_message>
<xml_diff>
--- a/Library/Library_Data/Data.xlsx
+++ b/Library/Library_Data/Data.xlsx
@@ -15,9 +15,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ h:mm:ss"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="2">
     <font>
       <name val="Calibri"/>
@@ -71,14 +69,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -457,20 +451,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22.85546875" customWidth="1" min="1" max="1"/>
-    <col width="24.140625" customWidth="1" min="2" max="2"/>
-    <col width="36.42578125" customWidth="1" min="3" max="3"/>
-    <col width="28.28515625" customWidth="1" min="4" max="4"/>
-    <col width="18.5703125" customWidth="1" min="5" max="5"/>
-    <col width="14.7109375" customWidth="1" min="6" max="6"/>
-    <col width="18.5703125" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="18.42578125" customWidth="1" min="2" max="2"/>
+    <col width="24.140625" customWidth="1" min="3" max="3"/>
+    <col width="36.42578125" customWidth="1" min="4" max="4"/>
+    <col width="28.28515625" customWidth="1" min="5" max="5"/>
+    <col width="18.5703125" customWidth="1" min="6" max="7"/>
     <col width="18.28515625" bestFit="1" customWidth="1" min="8" max="8"/>
     <col width="14.85546875" customWidth="1" min="9" max="9"/>
     <col width="13.85546875" customWidth="1" min="10" max="10"/>
-    <col width="10.85546875" customWidth="1" min="11" max="11"/>
+    <col width="15.28515625" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -481,27 +474,27 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Phone Number</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Unique code Of Book</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Name Of Book</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Author Of Book</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Price Of Book</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Quantity</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -533,138 +526,99 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Mayuresh Jagtap</t>
+          <t>Nitin Menon</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>MYTH10005</t>
+          <t>8798000000</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Shiva to Shankara</t>
+          <t>ROMNC10005</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Devdutt Pattanaik</t>
-        </is>
-      </c>
-      <c r="E2" t="n">
-        <v>275</v>
+          <t>The 3 Mistakes of My Life</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Chetan Bhagat</t>
+        </is>
       </c>
       <c r="F2" t="n">
-        <v>9</v>
+        <v>199</v>
       </c>
       <c r="G2" t="n">
-        <v>11</v>
-      </c>
-      <c r="H2" s="2" t="n">
-        <v>46265</v>
-      </c>
-      <c r="I2" s="3" t="n">
-        <v>25</v>
-      </c>
-      <c r="J2" s="2" t="n">
-        <v>46290.61308128472</v>
+        <v>8</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>01-09-2026</t>
+        </is>
+      </c>
+      <c r="I2" t="n">
+        <v>5</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>06-09-2026</t>
+        </is>
       </c>
       <c r="K2" t="n">
-        <v>99</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Manish Patel</t>
+          <t>Aman Patel</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>NOV10009</t>
+          <t>7587120000</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>The Lowland</t>
+          <t>NOV10010</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Jhumpa Lahiri</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
-        <v>399</v>
+          <t>Sea of Poppies</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Amitav Ghosh</t>
+        </is>
       </c>
       <c r="F3" t="n">
-        <v>1</v>
+        <v>450</v>
       </c>
       <c r="G3" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>31-08-2026</t>
+          <t>01-09-2026</t>
         </is>
       </c>
       <c r="I3" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>12-09-2026</t>
+          <t>11-09-2026</t>
         </is>
       </c>
       <c r="K3" t="n">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Aman Sharma</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>NOV10007</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Clear Light of Day</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Anita Desai</t>
-        </is>
-      </c>
-      <c r="E4" t="n">
-        <v>320</v>
-      </c>
-      <c r="F4" t="n">
-        <v>2</v>
-      </c>
-      <c r="G4" t="n">
-        <v>13</v>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>31-08-2026</t>
-        </is>
-      </c>
-      <c r="I4" t="n">
-        <v>6</v>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>06-09-2026</t>
-        </is>
-      </c>
-      <c r="K4" t="n">
-        <v>26</v>
+        <v>180</v>
       </c>
     </row>
   </sheetData>

</xml_diff>